<commit_message>
stop candidate mass upload features
</commit_message>
<xml_diff>
--- a/Documents/candidate-massupload-filled.xlsx
+++ b/Documents/candidate-massupload-filled.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Default.LAPTOP-9IUDD7TA\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90809B85-6D95-4BB9-BE85-2DBA85E29B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{897D5C11-0925-4CE1-97EE-7962278B4DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27456" yWindow="3012" windowWidth="16152" windowHeight="8208" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="75">
   <si>
     <t>FirstName</t>
   </si>
@@ -40,12 +40,6 @@
     <t>PositionApplied</t>
   </si>
   <si>
-    <t>CompanyCode</t>
-  </si>
-  <si>
-    <t>DivisionCode</t>
-  </si>
-  <si>
     <t>ExpectedSalary</t>
   </si>
   <si>
@@ -67,12 +61,6 @@
     <t>Software Developer</t>
   </si>
   <si>
-    <t>ULI</t>
-  </si>
-  <si>
-    <t>IT</t>
-  </si>
-  <si>
     <t>45000</t>
   </si>
   <si>
@@ -91,9 +79,6 @@
     <t>Business Analyst</t>
   </si>
   <si>
-    <t>BPM</t>
-  </si>
-  <si>
     <t>50000</t>
   </si>
   <si>
@@ -136,9 +121,6 @@
     <t>HR Specialist</t>
   </si>
   <si>
-    <t>HR</t>
-  </si>
-  <si>
     <t>38000</t>
   </si>
   <si>
@@ -181,9 +163,6 @@
     <t>Finance Analyst</t>
   </si>
   <si>
-    <t>FIN</t>
-  </si>
-  <si>
     <t>42000</t>
   </si>
   <si>
@@ -205,9 +184,6 @@
     <t>Project Coordinator</t>
   </si>
   <si>
-    <t>OPS</t>
-  </si>
-  <si>
     <t>Patricia</t>
   </si>
   <si>
@@ -224,9 +200,6 @@
   </si>
   <si>
     <t>Procurement Officer</t>
-  </si>
-  <si>
-    <t>SCM</t>
   </si>
   <si>
     <t>39000</t>
@@ -643,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
@@ -652,14 +625,12 @@
     <col min="4" max="4" width="22.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.90625" customWidth="1"/>
     <col min="6" max="6" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -681,301 +652,235 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B3" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="E3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="F3" t="s">
+      <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="E4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="F4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="G4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="D5" t="s">
         <v>30</v>
       </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="E5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="F5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>34</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
         <v>35</v>
       </c>
-      <c r="E5" t="s">
+      <c r="C6" t="s">
         <v>36</v>
       </c>
-      <c r="F5" t="s">
+      <c r="D6" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="I5" t="s">
+      <c r="F6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>41</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
         <v>42</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C7" t="s">
         <v>43</v>
       </c>
-      <c r="E6" t="s">
+      <c r="D7" t="s">
         <v>44</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E7" t="s">
         <v>45</v>
       </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="F7" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="G7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B8" t="s">
         <v>49</v>
       </c>
-      <c r="D7" t="s">
+      <c r="C8" t="s">
         <v>50</v>
       </c>
-      <c r="E7" t="s">
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="F7" t="s">
+      <c r="E8" t="s">
         <v>52</v>
       </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="F8" t="s">
         <v>53</v>
       </c>
-      <c r="I7" t="s">
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B9" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C9" t="s">
         <v>56</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E9" t="s">
         <v>58</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F9" t="s">
         <v>59</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G9" t="s">
         <v>60</v>
       </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>61</v>
       </c>
-      <c r="I8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B10" t="s">
         <v>62</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C10" t="s">
         <v>63</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D10" t="s">
         <v>64</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E10" t="s">
         <v>65</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F10" t="s">
         <v>66</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G10" t="s">
         <v>67</v>
       </c>
-      <c r="G9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>68</v>
       </c>
-      <c r="I9" t="s">
+      <c r="B11" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="C11" t="s">
         <v>70</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D11" t="s">
         <v>71</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E11" t="s">
         <v>72</v>
       </c>
-      <c r="D10" t="s">
+      <c r="F11" t="s">
         <v>73</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G11" t="s">
         <v>74</v>
-      </c>
-      <c r="F10" t="s">
-        <v>75</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" t="s">
-        <v>81</v>
-      </c>
-      <c r="F11" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>